<commit_message>
case_daily: fn<6 fix + BANK Jul29 retrofix + tape spec
- fn logic: thay fn_n=="1" bằng int(fn_n)<6 or low_conf=="True"
- taker (col5): luôn native, bỏ Zone-A substitution
- ratio cols {15,16,17}: ghi native + comment SUSPECT fn<6 khi fn_suspect
- PermissionError → raise RuntimeError [L-34], bỏ fallback _NEW file
- xóa _load_zone_a (dead code)
- CASE_BANK.xlsx Jul29 retrofix: taker 0.5046→0.4989 native, SUSPECT comment trên pos_r/acc_r/gLSR
- proposals/tape_daemon_spec.md: BR one-shot viable, daemon spec cho volume cao

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANK.xlsx
+++ b/docs/case_files/CASE_BANK.xlsx
@@ -426,9 +426,19 @@
     <author>case_daily.py</author>
   </authors>
   <commentList>
-    <comment ref="E37" authorId="0" shapeId="0">
+    <comment ref="O37" authorId="0" shapeId="0">
       <text>
-        <t>fn=1 (native_1d) — taker từ Zone-A-agg (ledger_v2 CAMPAIGNS/BANK_20260720)</t>
+        <t>SUSPECT fn&lt;6 (fn=1, src=native_1d)</t>
+      </text>
+    </comment>
+    <comment ref="P37" authorId="0" shapeId="0">
+      <text>
+        <t>SUSPECT fn&lt;6 (fn=1, src=native_1d)</t>
+      </text>
+    </comment>
+    <comment ref="Q37" authorId="0" shapeId="0">
+      <text>
+        <t>SUSPECT fn&lt;6 (fn=1, src=native_1d)</t>
       </text>
     </comment>
   </commentList>
@@ -3366,8 +3376,8 @@
         <f>IFERROR(B37/B36-1,"")</f>
         <v/>
       </c>
-      <c r="E37" t="n">
-        <v>0.5046</v>
+      <c r="E37" s="27" t="n">
+        <v>0.4989226837701057</v>
       </c>
       <c r="F37" s="27" t="n">
         <v>-0.00026779</v>

</xml_diff>

<commit_message>
fix export timing + re-generate 28-31/07 DAILY + L-41
- scripts/export_freshwatch_daily_vps.py: exclude today D from default dates
  (range 2..1 thay vi 2..0), them --force-regen strip+rebuild existing rows
- scripts/case_daily.py: them --force-overwrite overwrite SUSPECT hoac fn<6;
  fix MergedCell skip; them _row_fn_low() helper
- CASE_IDOL/TAG/BR/BANK.xlsx: DAILY 28-31/07 overwritten/appended,
  fn=1 cleared, px/vol filled tu native_1d store
- CASE_INDEX.xlsx LESSONS: L-41 append (timing rule)
- docs/lessons_learned.md: regenerate (41 bai hoc)
- agent_log.md: C1-C5 session log

CẦN OPERATOR: CASE_TAG.xlsx A32:L32 merged → TAG 30/07 fn/px chua ghi.
Unmerge A32:L32 roi chay: python scripts/case_daily.py --date 2026-07-30 --force-overwrite

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANK.xlsx
+++ b/docs/case_files/CASE_BANK.xlsx
@@ -418,31 +418,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>case_daily.py</author>
-  </authors>
-  <commentList>
-    <comment ref="O37" authorId="0" shapeId="0">
-      <text>
-        <t>SUSPECT fn&lt;6 (fn=1, src=native_1d)</t>
-      </text>
-    </comment>
-    <comment ref="P37" authorId="0" shapeId="0">
-      <text>
-        <t>SUSPECT fn&lt;6 (fn=1, src=native_1d)</t>
-      </text>
-    </comment>
-    <comment ref="Q37" authorId="0" shapeId="0">
-      <text>
-        <t>SUSPECT fn&lt;6 (fn=1, src=native_1d)</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -780,7 +755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AO37"/>
+  <dimension ref="A1:AO39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="27" min="1" max="1"/>
@@ -3372,27 +3347,33 @@
           <t>2026-07-29</t>
         </is>
       </c>
+      <c r="B37" s="27" t="n">
+        <v>0.1713490368477554</v>
+      </c>
       <c r="C37" s="27">
         <f>IFERROR(B37/B36-1,"")</f>
         <v/>
       </c>
+      <c r="D37" s="27" t="n">
+        <v>738355605.75427</v>
+      </c>
       <c r="E37" s="27" t="n">
         <v>0.4989226837701057</v>
       </c>
       <c r="F37" s="27" t="n">
-        <v>-0.00026779</v>
+        <v>-0.000988205</v>
       </c>
       <c r="G37" s="27" t="n">
-        <v>-0.00026779</v>
+        <v>-0.00205082</v>
       </c>
       <c r="H37" s="27" t="n">
-        <v>-0.00026779</v>
+        <v>-1.461e-05</v>
       </c>
       <c r="I37" s="27" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L37" s="27" t="n">
-        <v>25000000</v>
+        <v>25365666.16605</v>
       </c>
       <c r="O37" s="27" t="n">
         <v>1.3307</v>
@@ -3425,6 +3406,142 @@
       </c>
       <c r="AJ37" s="27">
         <f>IF(OR(AB37="",D37="",D37=0),"",AB37/D37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B38" s="27" t="n">
+        <v>0.0887329722906726</v>
+      </c>
+      <c r="C38" s="27">
+        <f>IFERROR(B38/B37-1,"")</f>
+        <v/>
+      </c>
+      <c r="D38" s="27" t="n">
+        <v>1039593900.21891</v>
+      </c>
+      <c r="E38" s="27" t="n">
+        <v>0.491663277755185</v>
+      </c>
+      <c r="F38" s="27" t="n">
+        <v>-0.003337582</v>
+      </c>
+      <c r="G38" s="27" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="H38" s="27" t="n">
+        <v>-4.97e-05</v>
+      </c>
+      <c r="I38" s="27" t="n">
+        <v>15</v>
+      </c>
+      <c r="L38" s="27" t="n">
+        <v>21421641.72207464</v>
+      </c>
+      <c r="O38" s="27" t="n">
+        <v>1.1134</v>
+      </c>
+      <c r="P38" s="27" t="n">
+        <v>0.9346</v>
+      </c>
+      <c r="Q38" s="27" t="n">
+        <v>0.9873</v>
+      </c>
+      <c r="R38" s="27">
+        <f>IFERROR(O38/P38,"")</f>
+        <v/>
+      </c>
+      <c r="S38" s="27">
+        <f>IFERROR(AVERAGE(R36:R38),"")</f>
+        <v/>
+      </c>
+      <c r="T38" s="27">
+        <f>IFERROR(Q38/Q33,"")</f>
+        <v/>
+      </c>
+      <c r="U38" s="27">
+        <f>IFERROR(O38/O35-1,"")</f>
+        <v/>
+      </c>
+      <c r="V38" s="27">
+        <f>IFERROR(P38/P35-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ38" s="27">
+        <f>IF(OR(AB38="",D38="",D38=0),"",AB38/D38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.0630603801681764</v>
+      </c>
+      <c r="C39">
+        <f>IFERROR(B39/B38-1,"")</f>
+        <v/>
+      </c>
+      <c r="D39" t="n">
+        <v>562696137.64149</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.491559894244458</v>
+      </c>
+      <c r="F39" t="n">
+        <v>-0.001911111666666667</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-0.00438872</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-0.00069484</v>
+      </c>
+      <c r="I39" t="n">
+        <v>24</v>
+      </c>
+      <c r="L39" t="n">
+        <v>17254036.24131712</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1.1095</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1.7933</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>1.5013</v>
+      </c>
+      <c r="R39">
+        <f>IFERROR(O39/P39,"")</f>
+        <v/>
+      </c>
+      <c r="S39">
+        <f>IFERROR(AVERAGE(R37:R39),"")</f>
+        <v/>
+      </c>
+      <c r="T39">
+        <f>IFERROR(Q39/Q34,"")</f>
+        <v/>
+      </c>
+      <c r="U39">
+        <f>IFERROR(O39/O36-1,"")</f>
+        <v/>
+      </c>
+      <c r="V39">
+        <f>IFERROR(P39/P36-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ39">
+        <f>IF(OR(AB39="",D39="",D39=0),"",AB39/D39)</f>
         <v/>
       </c>
     </row>
@@ -3438,7 +3555,6 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
BANK H1/H2/H3/H4: verify px_max + VWAP exit + CASE update (04/08)
H1: px_max SỬA — native 1h high = 0.67205 (27/07 06:00 UTC spike, 299M USDT vol).
    Trước dùng 0.37632 = daily avg 26/07, không phải intraday high.
    pos_r flat 1.30-1.36 trong khi px +42.7% (23-27/07): XÁC NHẬN.
    gLSR slope flip bền vững: 28/07 (sau spike).
H2: OI PRE FLAT 4.3-4.7M. Explosion trong MARKUP (+22M trong 9 ngày).
    Funding PnL MM ước tính: $26K-$43K (nhỏ, PnL chủ đạo = giá).
H3: Build VWAP=0.03943, Exit VWAP=0.19710. MM multiple THỰC=5.0× (+400%).
    Holder giấy: +897% (daily avg basis) / +1681% (spike high basis).
H4: CASE_BANK.xlsx CASE sheet — 17 machine rows append.
    OUTCOME T+14 (24/07): px=0.28339, ret=+651.1%, OI=51.12M, gLSR=0.500.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANK.xlsx
+++ b/docs/case_files/CASE_BANK.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="169" formatCode="0.000"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -96,8 +96,11 @@
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -152,6 +155,11 @@
         <bgColor rgb="FF375623"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4A843"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -187,7 +195,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -348,6 +356,7 @@
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -601,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="27" min="1" max="1"/>
@@ -739,6 +748,216 @@
       <c r="B14" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">O vang = operator dien/quyet · Header nau vang (sheet DAILY) = cot manual · Dong to cam (DAILY) = data_bad=1, so mang sai so · Cot cong thuc (ret_1d, div, slope, oi_vs_med14, alpha) tu tinh khi may append dong moi — copy cong thuc dong tren xuong. </t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54">
+        <f>== PROBE-VERIFIED — H1/H2/H3 (04/08/2026) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>px_T0 probe-verified</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0.03773 (freshwatch 10/07 px_avg)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>px_max [1h spike native]</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.67205 USDT — 27/07 06:00 UTC (fapi 1h high, vol 299M USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>px_max [daily avg basis]</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0.37632 USDT — 26/07 freshwatch avg (truoc da dung lam px_max)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>px_max [close basis]</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0.41958 USDT — 27/07 close (fapi 1h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>markup T0→spike_high</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>+1681% (0.03773→0.67205)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>markup T0→daily_avg_max</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>+897% (0.03773→0.37632)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>OI PRE range (25/06-09/07)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>4.31M→4.73M FLAT — khong xay duoc truoc markup</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>OI MARKUP peak (19/07)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>26.56M USD (tu 4.47M T0: +22M trong 9 ngay)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MM_build_VWAP</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0.03943 USDT (daily 25/06-12/07 approx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MM_exit_VWAP</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0.19710 USDT (1h klines 19-21/07, pos_r sap window)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MM_multiple_thuc</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>5.00x (+400%) = exit_VWAP / build_VWAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>MM_funding_PnL_PRE_MARKUP</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>$26K-$43K total (27/06-19/07, 3-5M long, khong dang ke)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>gLSR_min_POST</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0.390 — 20/07 (ngay sau pos_r crash)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>gLSR_slope_flip_sustained</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>28/07 (sau spike 27/07) — da tang lien tuc len 1.726 ngay 03/08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>pos_r_flat_window</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1.30-1.36 (23-27/07) — khi px tang 0.247→0.376 (+42.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>pos_r_crash_window</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>19-20/07: 1.61→1.09 (MM phan phoi trong khi px van tang)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>_probe_bank_h1h2h3_20260804.py run 04/08/2026</t>
         </is>
       </c>
     </row>
@@ -3478,69 +3697,69 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="27" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="27" t="n">
         <v>0.0630603801681764</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="27">
         <f>IFERROR(B39/B38-1,"")</f>
         <v/>
       </c>
-      <c r="D39" t="n">
+      <c r="D39" s="27" t="n">
         <v>562696137.64149</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="27" t="n">
         <v>0.491559894244458</v>
       </c>
-      <c r="F39" t="n">
+      <c r="F39" s="27" t="n">
         <v>-0.001911111666666667</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G39" s="27" t="n">
         <v>-0.00438872</v>
       </c>
-      <c r="H39" t="n">
+      <c r="H39" s="27" t="n">
         <v>-0.00069484</v>
       </c>
-      <c r="I39" t="n">
+      <c r="I39" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="L39" t="n">
+      <c r="L39" s="27" t="n">
         <v>17254036.24131712</v>
       </c>
-      <c r="O39" t="n">
+      <c r="O39" s="27" t="n">
         <v>1.1095</v>
       </c>
-      <c r="P39" t="n">
+      <c r="P39" s="27" t="n">
         <v>1.7933</v>
       </c>
-      <c r="Q39" t="n">
+      <c r="Q39" s="27" t="n">
         <v>1.5013</v>
       </c>
-      <c r="R39">
+      <c r="R39" s="27">
         <f>IFERROR(O39/P39,"")</f>
         <v/>
       </c>
-      <c r="S39">
+      <c r="S39" s="27">
         <f>IFERROR(AVERAGE(R37:R39),"")</f>
         <v/>
       </c>
-      <c r="T39">
+      <c r="T39" s="27">
         <f>IFERROR(Q39/Q34,"")</f>
         <v/>
       </c>
-      <c r="U39">
+      <c r="U39" s="27">
         <f>IFERROR(O39/O36-1,"")</f>
         <v/>
       </c>
-      <c r="V39">
+      <c r="V39" s="27">
         <f>IFERROR(P39/P36-1,"")</f>
         <v/>
       </c>
-      <c r="AJ39">
+      <c r="AJ39" s="27">
         <f>IF(OR(AB39="",D39="",D39=0),"",AB39/D39)</f>
         <v/>
       </c>
@@ -3900,6 +4119,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="53" t="inlineStr">
         <is>
@@ -3958,12 +4178,30 @@
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="C4" s="33" t="n"/>
-      <c r="D4" s="33" t="n"/>
-      <c r="E4" s="33" t="n"/>
-      <c r="F4" s="33" t="n"/>
-      <c r="G4" s="33" t="n"/>
-      <c r="H4" s="33" t="n"/>
+      <c r="C4" s="33" t="n">
+        <v>0.28339</v>
+      </c>
+      <c r="D4" s="33" t="inlineStr">
+        <is>
+          <t>+651.1%</t>
+        </is>
+      </c>
+      <c r="E4" s="33" t="inlineStr">
+        <is>
+          <t>peak→down</t>
+        </is>
+      </c>
+      <c r="F4" s="33" t="n">
+        <v>51120000</v>
+      </c>
+      <c r="G4" s="33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H4" s="33" t="inlineStr">
+        <is>
+          <t>px van cao (24/07 avg 0.283), OI 51M, gLSR 0.500 — POST dang sap</t>
+        </is>
+      </c>
       <c r="I4" s="33" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="28">

</xml_diff>

<commit_message>
BANK J2/J3/J4: June chain + unlock cadence + CASE update (04/08)
J2: fapi 1d klines + fundingRate 180 periods tháng 6. freshwatch 6 rows (09/06, 13/06, 27-30/06).
J3(a): 17/06 unlock QUIET (1.6M vol). Pump thực ở 05-08/06 (T-9): 50M vol + funding burst 23.4bps.
J3(b): Ngày bất thường #1 = 07/06 (50.9M USDT), không phải quanh unlock.
J3(c): acc_r=0.952 ngày 13/06 (T-27). Lead-time thực ≥T-31, không phải T-11 calib.
J3(d): Funding pin từ ≥01/05. Breaks mới: 08/06 và 11/06 (chưa có trong hồ sơ cũ).
J3(e): Jun vs Jul = KHÔNG lặp cấu trúc (vol 1×  vs 1076×). Vân tay #5 CHƯA ĐỦ bằng chứng.
J4: CASE_BANK UNLOCK calendar + 4 EVENTS rows + OUTCOME px_max spike note.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANK.xlsx
+++ b/docs/case_files/CASE_BANK.xlsx
@@ -195,7 +195,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -357,6 +357,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -758,204 +759,204 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>px_T0 probe-verified</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>0.03773 (freshwatch 10/07 px_avg)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>px_max [1h spike native]</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>0.67205 USDT — 27/07 06:00 UTC (fapi 1h high, vol 299M USDT)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>px_max [daily avg basis]</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>0.37632 USDT — 26/07 freshwatch avg (truoc da dung lam px_max)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>px_max [close basis]</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>0.41958 USDT — 27/07 close (fapi 1h)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>markup T0→spike_high</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>+1681% (0.03773→0.67205)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="27" t="inlineStr">
         <is>
           <t>markup T0→daily_avg_max</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>+897% (0.03773→0.37632)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t>OI PRE range (25/06-09/07)</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>4.31M→4.73M FLAT — khong xay duoc truoc markup</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>OI MARKUP peak (19/07)</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>26.56M USD (tu 4.47M T0: +22M trong 9 ngay)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="27" t="inlineStr">
         <is>
           <t>MM_build_VWAP</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>0.03943 USDT (daily 25/06-12/07 approx)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>MM_exit_VWAP</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>0.19710 USDT (1h klines 19-21/07, pos_r sap window)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="27" t="inlineStr">
         <is>
           <t>MM_multiple_thuc</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="27" t="inlineStr">
         <is>
           <t>5.00x (+400%) = exit_VWAP / build_VWAP</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>MM_funding_PnL_PRE_MARKUP</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>$26K-$43K total (27/06-19/07, 3-5M long, khong dang ke)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="27" t="inlineStr">
         <is>
           <t>gLSR_min_POST</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>0.390 — 20/07 (ngay sau pos_r crash)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="27" t="inlineStr">
         <is>
           <t>gLSR_slope_flip_sustained</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>28/07 (sau spike 27/07) — da tang lien tuc len 1.726 ngay 03/08)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="27" t="inlineStr">
         <is>
           <t>pos_r_flat_window</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>1.30-1.36 (23-27/07) — khi px tang 0.247→0.376 (+42.7%)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="27" t="inlineStr">
         <is>
           <t>pos_r_crash_window</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="27" t="inlineStr">
         <is>
           <t>19-20/07: 1.61→1.09 (MM phan phoi trong khi px van tang)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="27" t="inlineStr">
         <is>
           <t>SOURCE</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="27" t="inlineStr">
         <is>
           <t>_probe_bank_h1h2h3_20260804.py run 04/08/2026</t>
         </is>
@@ -3783,7 +3784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="27" min="1" max="1"/>
@@ -3972,6 +3973,94 @@
       <c r="D10" s="32" t="inlineStr">
         <is>
           <t>phan phoi hau-dinh, suppressor dung</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06-05/06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>mini-pump: vol 10M→25M→50.9M→41M (05-08/06), high 0.045, funding BURST 08/06 (23.4bps peak). Flush down 05/06 (low 0.022), recover 06-08/06. T-10 so với 17/06 unlock.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>fapi klines + fundingRate (probe 04/08)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>bait-probe trước unlock Jun? (vol+funding chỉ dấu)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06-17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Unlock ~2% supply 17/06: QUIET (vol 1.6M, px ~0.04). Funding toàn PIN. Sau unlock: px -8% đến 22/06. acc_r=0.952 ngày 13/06 (ĐÃ CAO TRƯỚC UNLOCK).</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>fapi klines + freshwatch 09/06+13/06 (probe 04/08)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>unlock không kèm markup — đè sau để gom rẻ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07-17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Unlock ~2% supply 17/07: TRONG đỉnh markup. px=0.068 (T+7). MM XẢ T+2→T+4 (19-21/07): pos_r 3.7→1.09, vol 1.4-6.5B/ngày. Khuôn L-12: kéo-trước-xả-vào-hype sau unlock.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>freshwatch + calib (probe 04/08)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>unlock = mốc xả MM; vol unlock = thanh khoản thoát</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07-27 06:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>px_max SPIKE 0.67205 USDT (1h native fapi). vol 299.72M USDT trong 1 nến. Close 0.419. Freshwatch daily avg 27/07=0.374. Wick spike — không phải close-based peak. px_max trước ghi 0.376 = WRONG.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>fapi 1h klines (probe H1 04/08)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>px_max thực = 0.672 spike, không phải 0.376 daily avg</t>
         </is>
       </c>
     </row>
@@ -4099,7 +4188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="27" min="1" max="1"/>
@@ -4188,7 +4277,7 @@
       </c>
       <c r="E4" s="33" t="inlineStr">
         <is>
-          <t>peak→down</t>
+          <t>spike_high=0.672 ngày 27/07 (wick); close_max=0.419; daily_avg_max=0.376 (26/07)</t>
         </is>
       </c>
       <c r="F4" s="33" t="n">
@@ -4241,6 +4330,18 @@
       <c r="G6" s="33" t="n"/>
       <c r="H6" s="33" t="n"/>
       <c r="I6" s="33" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>px_max SỬA (probe H1 04/08): 1h spike high = 0.67205 (27/07 06:00 UTC, 299M USDT). Daily avg max = 0.37632 (26/07 freshwatch). Close max = 0.41958 (27/07). Markup từ T0 (0.03773): +1681% spike / +897% daily avg / +1012% close.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -4390,7 +4491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="27" min="1" max="1"/>
@@ -4404,6 +4505,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="31" t="inlineStr">
         <is>
@@ -4412,7 +4514,7 @@
       </c>
       <c r="B3" s="33" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>PENDING (operator feed)</t>
         </is>
       </c>
     </row>
@@ -4424,7 +4526,7 @@
       </c>
       <c r="B4" s="33" t="inlineStr">
         <is>
-          <t>PENDING (CryptoRank/TokenUnlocks)</t>
+          <t>operator 04/08/2026 — CryptoRank/TokenUnlocks</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4538,7 @@
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>17/08/2026 (T+38 từ T0 10/07) — ~2% supply/tháng</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4550,7 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>17/08 · 17/09 · 17/10 (~2%/tháng mỗi lần)</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4562,7 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>17/07/2026 — KHỚP exact với exit window 19-21/07 (T+7→T+9)</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4574,49 @@
       </c>
       <c r="B8" s="33" t="inlineStr">
         <is>
-          <t>PENDING — viec tay #3 tracker</t>
+          <t>Khuôn L-12: MM xả T+2→T+4 sau unlock 17/07. Cảnh báo 17/08.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="55">
+        <f>== UNLOCK CALENDAR (operator 04/08) ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>17/06/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>[PAST] Quanh 17/06: KHÔNG có markup. Trước đó 05-08/06 vol spike 50M→41M (mini-pump T-10 đến T-9). Funding BURST 08/06 (23.4bps). Unlock chính ngày 17/06 = QUIET (vol 1.6M). Sau 17/06: px giảm -8% đến 22/06. Pattern = đè-sau-unlock (chưa campaign).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>17/07/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>[PAST — KHỚP CAMPAIGN] Unlock T+7 từ T0 (10/07). Trong đỉnh markup (+280% đến ngày này). MM XẢ T+2→T+4 sau unlock: pos_r 3.7→1.09 (19-21/07). KẾT LUẬN: unlock là mốc xả — MM dùng vol unlock làm thanh khoản thoát.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>[UPCOMING — T+38 từ T0] CẢNH BÁO: token đang SUPPRESSED (px 0.043 = -93.6% từ spike 0.672). Nếu khuôn lặp: cửa sổ bait = 02/08→17/08. NHƯNG: pos_r chưa reset, không có bằng chứng MM build mới. → Theo dõi như RỦI RO (không phải cơ hội). Operator quyết.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BANK spot audit W1-W5: venue map + daily series 01/07->05/08 + P8 verdict
- Xac nhan BANKUSDT co listing Binance spot (36 ngay du lieu, vol $0.1-124M/ngay)
- Alpha ALPHA_146: endpoint 400 — ABSTAIN; BSC DEX: nho ($14K/day max)
- Spot/perp ratio campaign avg 0.113x, peak week avg 0.067x (bi gau boi perp vol)
- Taker spot peak week (vol-weighted): 51.2% -> NEUTRAL -> P8 AMBIGUOUS
- 80M tokens at peak px = ~$20M / $598M spot vol = 3% -> khong phat hien duoc tu taker
- CASE_BANK DAILY spot cols (venue/vol_spot/taker_spot): fill 31 ngay 01/07->04/08
- T+30 = 09/08: px_now 0.052 vs advisor_exit VWAP 0.197 = -73.4%
- Probe archived: scripts/archive/_probe_bank_spot_20260805.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANK.xlsx
+++ b/docs/case_files/CASE_BANK.xlsx
@@ -195,7 +195,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -358,6 +358,8 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1714,6 +1716,17 @@
         <f>IFERROR(P9/P6-1,"")</f>
         <v/>
       </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB9" s="56" t="n">
+        <v>286000</v>
+      </c>
+      <c r="AC9" s="57" t="n">
+        <v>0.67</v>
+      </c>
       <c r="AJ9" s="27">
         <f>IF(OR(AB9="",D9="",D9=0),"",AB9/D9)</f>
         <v/>
@@ -1782,6 +1795,17 @@
         <f>IFERROR(P10/P7-1,"")</f>
         <v/>
       </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB10" s="56" t="n">
+        <v>3750000</v>
+      </c>
+      <c r="AC10" s="57" t="n">
+        <v>0.512</v>
+      </c>
       <c r="AJ10" s="27">
         <f>IF(OR(AB10="",D10="",D10=0),"",AB10/D10)</f>
         <v/>
@@ -1850,6 +1874,17 @@
         <f>IFERROR(P11/P8-1,"")</f>
         <v/>
       </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB11" s="56" t="n">
+        <v>397000</v>
+      </c>
+      <c r="AC11" s="57" t="n">
+        <v>0.363</v>
+      </c>
       <c r="AJ11" s="27">
         <f>IF(OR(AB11="",D11="",D11=0),"",AB11/D11)</f>
         <v/>
@@ -1918,6 +1953,17 @@
         <f>IFERROR(P12/P9-1,"")</f>
         <v/>
       </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB12" s="56" t="n">
+        <v>203000</v>
+      </c>
+      <c r="AC12" s="57" t="n">
+        <v>0.376</v>
+      </c>
       <c r="AJ12" s="27">
         <f>IF(OR(AB12="",D12="",D12=0),"",AB12/D12)</f>
         <v/>
@@ -1986,6 +2032,17 @@
         <f>IFERROR(P13/P10-1,"")</f>
         <v/>
       </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB13" s="56" t="n">
+        <v>243000</v>
+      </c>
+      <c r="AC13" s="57" t="n">
+        <v>0.527</v>
+      </c>
       <c r="AJ13" s="27">
         <f>IF(OR(AB13="",D13="",D13=0),"",AB13/D13)</f>
         <v/>
@@ -2054,6 +2111,17 @@
         <f>IFERROR(P14/P11-1,"")</f>
         <v/>
       </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB14" s="56" t="n">
+        <v>230000</v>
+      </c>
+      <c r="AC14" s="57" t="n">
+        <v>0.507</v>
+      </c>
       <c r="AJ14" s="27">
         <f>IF(OR(AB14="",D14="",D14=0),"",AB14/D14)</f>
         <v/>
@@ -2122,6 +2190,17 @@
         <f>IFERROR(P15/P12-1,"")</f>
         <v/>
       </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB15" s="56" t="n">
+        <v>491000</v>
+      </c>
+      <c r="AC15" s="57" t="n">
+        <v>0.455</v>
+      </c>
       <c r="AJ15" s="27">
         <f>IF(OR(AB15="",D15="",D15=0),"",AB15/D15)</f>
         <v/>
@@ -2190,6 +2269,17 @@
         <f>IFERROR(P16/P13-1,"")</f>
         <v/>
       </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB16" s="56" t="n">
+        <v>530000</v>
+      </c>
+      <c r="AC16" s="57" t="n">
+        <v>0.543</v>
+      </c>
       <c r="AJ16" s="27">
         <f>IF(OR(AB16="",D16="",D16=0),"",AB16/D16)</f>
         <v/>
@@ -2258,6 +2348,17 @@
         <f>IFERROR(P17/P14-1,"")</f>
         <v/>
       </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB17" s="56" t="n">
+        <v>131000</v>
+      </c>
+      <c r="AC17" s="57" t="n">
+        <v>0.426</v>
+      </c>
       <c r="AJ17" s="27">
         <f>IF(OR(AB17="",D17="",D17=0),"",AB17/D17)</f>
         <v/>
@@ -2326,6 +2427,17 @@
         <f>IFERROR(P18/P15-1,"")</f>
         <v/>
       </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB18" s="56" t="n">
+        <v>675000</v>
+      </c>
+      <c r="AC18" s="57" t="n">
+        <v>0.433</v>
+      </c>
       <c r="AJ18" s="27">
         <f>IF(OR(AB18="",D18="",D18=0),"",AB18/D18)</f>
         <v/>
@@ -2394,6 +2506,17 @@
         <f>IFERROR(P19/P16-1,"")</f>
         <v/>
       </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB19" s="56" t="n">
+        <v>2440000</v>
+      </c>
+      <c r="AC19" s="57" t="n">
+        <v>0.477</v>
+      </c>
       <c r="AJ19" s="27">
         <f>IF(OR(AB19="",D19="",D19=0),"",AB19/D19)</f>
         <v/>
@@ -2462,6 +2585,17 @@
         <f>IFERROR(P20/P17-1,"")</f>
         <v/>
       </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB20" s="56" t="n">
+        <v>1610000</v>
+      </c>
+      <c r="AC20" s="57" t="n">
+        <v>0.437</v>
+      </c>
       <c r="AJ20" s="27">
         <f>IF(OR(AB20="",D20="",D20=0),"",AB20/D20)</f>
         <v/>
@@ -2530,6 +2664,17 @@
         <f>IFERROR(P21/P18-1,"")</f>
         <v/>
       </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB21" s="56" t="n">
+        <v>573000</v>
+      </c>
+      <c r="AC21" s="57" t="n">
+        <v>0.491</v>
+      </c>
       <c r="AJ21" s="27">
         <f>IF(OR(AB21="",D21="",D21=0),"",AB21/D21)</f>
         <v/>
@@ -2598,6 +2743,17 @@
         <f>IFERROR(P22/P19-1,"")</f>
         <v/>
       </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB22" s="56" t="n">
+        <v>459000</v>
+      </c>
+      <c r="AC22" s="57" t="n">
+        <v>0.605</v>
+      </c>
       <c r="AJ22" s="27">
         <f>IF(OR(AB22="",D22="",D22=0),"",AB22/D22)</f>
         <v/>
@@ -2666,6 +2822,17 @@
         <f>IFERROR(P23/P20-1,"")</f>
         <v/>
       </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB23" s="56" t="n">
+        <v>2460000</v>
+      </c>
+      <c r="AC23" s="57" t="n">
+        <v>0.53</v>
+      </c>
       <c r="AJ23" s="27">
         <f>IF(OR(AB23="",D23="",D23=0),"",AB23/D23)</f>
         <v/>
@@ -2734,6 +2901,17 @@
         <f>IFERROR(P24/P21-1,"")</f>
         <v/>
       </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB24" s="56" t="n">
+        <v>6400000</v>
+      </c>
+      <c r="AC24" s="57" t="n">
+        <v>0.518</v>
+      </c>
       <c r="AJ24" s="27">
         <f>IF(OR(AB24="",D24="",D24=0),"",AB24/D24)</f>
         <v/>
@@ -2802,6 +2980,17 @@
         <f>IFERROR(P25/P22-1,"")</f>
         <v/>
       </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB25" s="56" t="n">
+        <v>21450000</v>
+      </c>
+      <c r="AC25" s="57" t="n">
+        <v>0.497</v>
+      </c>
       <c r="AJ25" s="27">
         <f>IF(OR(AB25="",D25="",D25=0),"",AB25/D25)</f>
         <v/>
@@ -2870,6 +3059,17 @@
         <f>IFERROR(P26/P23-1,"")</f>
         <v/>
       </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB26" s="56" t="n">
+        <v>29800000</v>
+      </c>
+      <c r="AC26" s="57" t="n">
+        <v>0.528</v>
+      </c>
       <c r="AJ26" s="27">
         <f>IF(OR(AB26="",D26="",D26=0),"",AB26/D26)</f>
         <v/>
@@ -2938,6 +3138,17 @@
         <f>IFERROR(P27/P24-1,"")</f>
         <v/>
       </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB27" s="56" t="n">
+        <v>114270000</v>
+      </c>
+      <c r="AC27" s="57" t="n">
+        <v>0.522</v>
+      </c>
       <c r="AJ27" s="27">
         <f>IF(OR(AB27="",D27="",D27=0),"",AB27/D27)</f>
         <v/>
@@ -3006,6 +3217,17 @@
         <f>IFERROR(P28/P25-1,"")</f>
         <v/>
       </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB28" s="56" t="n">
+        <v>77060000</v>
+      </c>
+      <c r="AC28" s="57" t="n">
+        <v>0.528</v>
+      </c>
       <c r="AJ28" s="27">
         <f>IF(OR(AB28="",D28="",D28=0),"",AB28/D28)</f>
         <v/>
@@ -3074,6 +3296,17 @@
         <f>IFERROR(P29/P26-1,"")</f>
         <v/>
       </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB29" s="56" t="n">
+        <v>97030000</v>
+      </c>
+      <c r="AC29" s="57" t="n">
+        <v>0.499</v>
+      </c>
       <c r="AJ29" s="27">
         <f>IF(OR(AB29="",D29="",D29=0),"",AB29/D29)</f>
         <v/>
@@ -3142,6 +3375,17 @@
         <f>IFERROR(P30/P27-1,"")</f>
         <v/>
       </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB30" s="56" t="n">
+        <v>97100000</v>
+      </c>
+      <c r="AC30" s="57" t="n">
+        <v>0.509</v>
+      </c>
       <c r="AJ30" s="27">
         <f>IF(OR(AB30="",D30="",D30=0),"",AB30/D30)</f>
         <v/>
@@ -3210,6 +3454,17 @@
         <f>IFERROR(P31/P28-1,"")</f>
         <v/>
       </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB31" s="56" t="n">
+        <v>55960000</v>
+      </c>
+      <c r="AC31" s="57" t="n">
+        <v>0.505</v>
+      </c>
       <c r="AJ31" s="27">
         <f>IF(OR(AB31="",D31="",D31=0),"",AB31/D31)</f>
         <v/>
@@ -3278,6 +3533,17 @@
         <f>IFERROR(P32/P29-1,"")</f>
         <v/>
       </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB32" s="56" t="n">
+        <v>65500000</v>
+      </c>
+      <c r="AC32" s="57" t="n">
+        <v>0.507</v>
+      </c>
       <c r="AJ32" s="27">
         <f>IF(OR(AB32="",D32="",D32=0),"",AB32/D32)</f>
         <v/>
@@ -3346,6 +3612,17 @@
         <f>IFERROR(P33/P30-1,"")</f>
         <v/>
       </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB33" s="56" t="n">
+        <v>45180000</v>
+      </c>
+      <c r="AC33" s="57" t="n">
+        <v>0.511</v>
+      </c>
       <c r="AJ33" s="27">
         <f>IF(OR(AB33="",D33="",D33=0),"",AB33/D33)</f>
         <v/>
@@ -3419,6 +3696,17 @@
           <t>lsr_accum|stealth_grind|oi_ignition</t>
         </is>
       </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB34" s="56" t="n">
+        <v>35560000</v>
+      </c>
+      <c r="AC34" s="57" t="n">
+        <v>0.514</v>
+      </c>
       <c r="AJ34" s="27">
         <f>IF(OR(AB34="",D34="",D34=0),"",AB34/D34)</f>
         <v/>
@@ -3497,6 +3785,17 @@
           <t>lsr_accum|stealth_grind|oi_ignition</t>
         </is>
       </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB35" s="56" t="n">
+        <v>124750000</v>
+      </c>
+      <c r="AC35" s="57" t="n">
+        <v>0.517</v>
+      </c>
       <c r="AJ35" s="27">
         <f>IF(OR(AB35="",D35="",D35=0),"",AB35/D35)</f>
         <v/>
@@ -3551,6 +3850,17 @@
           <t>dist_wall|post_climax</t>
         </is>
       </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB36" s="56" t="n">
+        <v>116370000</v>
+      </c>
+      <c r="AC36" s="57" t="n">
+        <v>0.511</v>
+      </c>
       <c r="AJ36" s="27">
         <f>IF(OR(AB36="",D36="",D36=0),"",AB36/D36)</f>
         <v/>
@@ -3578,7 +3888,7 @@
         <v>738355605.75427</v>
       </c>
       <c r="E37" s="27" t="n">
-        <v>0.4989226837701057</v>
+        <v>49.892268</v>
       </c>
       <c r="F37" s="27" t="n">
         <v>-0.000988205</v>
@@ -3624,6 +3934,17 @@
         <f>IFERROR(P37/P34-1,"")</f>
         <v/>
       </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB37" s="56" t="n">
+        <v>66910000</v>
+      </c>
+      <c r="AC37" s="57" t="n">
+        <v>0.507</v>
+      </c>
       <c r="AJ37" s="27">
         <f>IF(OR(AB37="",D37="",D37=0),"",AB37/D37)</f>
         <v/>
@@ -3646,7 +3967,7 @@
         <v>1039593900.21891</v>
       </c>
       <c r="E38" s="27" t="n">
-        <v>0.491663277755185</v>
+        <v>49.166328</v>
       </c>
       <c r="F38" s="27" t="n">
         <v>-0.003337582</v>
@@ -3692,6 +4013,17 @@
         <f>IFERROR(P38/P35-1,"")</f>
         <v/>
       </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB38" s="56" t="n">
+        <v>85580000</v>
+      </c>
+      <c r="AC38" s="57" t="n">
+        <v>0.465</v>
+      </c>
       <c r="AJ38" s="27">
         <f>IF(OR(AB38="",D38="",D38=0),"",AB38/D38)</f>
         <v/>
@@ -3714,7 +4046,7 @@
         <v>562696137.64149</v>
       </c>
       <c r="E39" s="27" t="n">
-        <v>0.491559894244458</v>
+        <v>49.155989</v>
       </c>
       <c r="F39" s="27" t="n">
         <v>-0.001911111666666667</v>
@@ -3759,6 +4091,17 @@
       <c r="V39" s="27">
         <f>IFERROR(P39/P36-1,"")</f>
         <v/>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB39" s="56" t="n">
+        <v>35330000</v>
+      </c>
+      <c r="AC39" s="57" t="n">
+        <v>0.466</v>
       </c>
       <c r="AJ39" s="27">
         <f>IF(OR(AB39="",D39="",D39=0),"",AB39/D39)</f>
@@ -3977,88 +4320,88 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>06-05/06</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>mini-pump: vol 10M→25M→50.9M→41M (05-08/06), high 0.045, funding BURST 08/06 (23.4bps peak). Flush down 05/06 (low 0.022), recover 06-08/06. T-10 so với 17/06 unlock.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>fapi klines + fundingRate (probe 04/08)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>bait-probe trước unlock Jun? (vol+funding chỉ dấu)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>06-17</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>Unlock ~2% supply 17/06: QUIET (vol 1.6M, px ~0.04). Funding toàn PIN. Sau unlock: px -8% đến 22/06. acc_r=0.952 ngày 13/06 (ĐÃ CAO TRƯỚC UNLOCK).</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>fapi klines + freshwatch 09/06+13/06 (probe 04/08)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>unlock không kèm markup — đè sau để gom rẻ</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>07-17</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>Unlock ~2% supply 17/07: TRONG đỉnh markup. px=0.068 (T+7). MM XẢ T+2→T+4 (19-21/07): pos_r 3.7→1.09, vol 1.4-6.5B/ngày. Khuôn L-12: kéo-trước-xả-vào-hype sau unlock.</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>freshwatch + calib (probe 04/08)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>unlock = mốc xả MM; vol unlock = thanh khoản thoát</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="27" t="inlineStr">
         <is>
           <t>07-27 06:00</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>px_max SPIKE 0.67205 USDT (1h native fapi). vol 299.72M USDT trong 1 nến. Close 0.419. Freshwatch daily avg 27/07=0.374. Wick spike — không phải close-based peak. px_max trước ghi 0.376 = WRONG.</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>fapi 1h klines (probe H1 04/08)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="27" t="inlineStr">
         <is>
           <t>px_max thực = 0.672 spike, không phải 0.376 daily avg</t>
         </is>
@@ -4208,7 +4551,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="53" t="inlineStr">
         <is>
@@ -4332,12 +4674,12 @@
       <c r="I6" s="33" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>px_max SỬA (probe H1 04/08): 1h spike high = 0.67205 (27/07 06:00 UTC, 299M USDT). Daily avg max = 0.37632 (26/07 freshwatch). Close max = 0.41958 (27/07). Markup từ T0 (0.03773): +1681% spike / +897% daily avg / +1012% close.</t>
         </is>
@@ -4505,7 +4847,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="31" t="inlineStr">
         <is>
@@ -4585,36 +4926,36 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>17/06/2026</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>[PAST] Quanh 17/06: KHÔNG có markup. Trước đó 05-08/06 vol spike 50M→41M (mini-pump T-10 đến T-9). Funding BURST 08/06 (23.4bps). Unlock chính ngày 17/06 = QUIET (vol 1.6M). Sau 17/06: px giảm -8% đến 22/06. Pattern = đè-sau-unlock (chưa campaign).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>17/07/2026</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>[PAST — KHỚP CAMPAIGN] Unlock T+7 từ T0 (10/07). Trong đỉnh markup (+280% đến ngày này). MM XẢ T+2→T+4 sau unlock: pos_r 3.7→1.09 (19-21/07). KẾT LUẬN: unlock là mốc xả — MM dùng vol unlock làm thanh khoản thoát.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>17/08/2026</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>[UPCOMING — T+38 từ T0] CẢNH BÁO: token đang SUPPRESSED (px 0.043 = -93.6% từ spike 0.672). Nếu khuôn lặp: cửa sổ bait = 02/08→17/08. NHƯNG: pos_r chưa reset, không có bằng chứng MM build mới. → Theo dõi như RỦI RO (không phải cơ hội). Operator quyết.</t>
         </is>

</xml_diff>

<commit_message>
BANK vong-2 watch + OUTCOME T+30 + mm_econ v0.2
- CASE_BANK DAILY: append 5 rows 01-05/08 (freshwatch VPS + fapi)
  01-04/08 confirmed freshwatch; 05/08 data_bad=1 (partial)
  pos_r re-rate 1.11->1.32 nhung chua on dinh; gLSR peak 1.88 roi giam 1.40
- Nen 04/08 (+19% O->C): vol $471M, taker 49.1%, OI flat -> SHORT SQUEEZE, khong phai Ignition
- 3 dieu kien Vong 2: 0/3 thoa man (05/08) — funding van am, chua co pin duong moi
- CASE_BANK OUTCOME T+30 filled: px=0.0495, T0=0.0377, ret=+31.3%
  Tu +897% dinh ve +31% = full collapse; advisor exit VWAP 0.197 -> crowd -74.9%
- mm_econ v0.2: them cot kho_vol_ratio (BANK=2.6%), taker detection floor ~10% rule,
  M7 BANK Vong 2 watch, M6 detection floor methodology

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANK.xlsx
+++ b/docs/case_files/CASE_BANK.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="0.00000000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
@@ -30,6 +30,7 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="0.000"/>
     <numFmt numFmtId="170" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="0.00000"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -100,7 +101,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -160,6 +161,11 @@
         <fgColor rgb="00D4A843"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -195,7 +201,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -360,6 +366,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -977,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AO39"/>
+  <dimension ref="A1:AO44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="27" min="1" max="1"/>
@@ -1716,7 +1732,7 @@
         <f>IFERROR(P9/P6-1,"")</f>
         <v/>
       </c>
-      <c r="AA9" t="inlineStr">
+      <c r="AA9" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -1795,7 +1811,7 @@
         <f>IFERROR(P10/P7-1,"")</f>
         <v/>
       </c>
-      <c r="AA10" t="inlineStr">
+      <c r="AA10" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -1874,7 +1890,7 @@
         <f>IFERROR(P11/P8-1,"")</f>
         <v/>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="AA11" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -1953,7 +1969,7 @@
         <f>IFERROR(P12/P9-1,"")</f>
         <v/>
       </c>
-      <c r="AA12" t="inlineStr">
+      <c r="AA12" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2032,7 +2048,7 @@
         <f>IFERROR(P13/P10-1,"")</f>
         <v/>
       </c>
-      <c r="AA13" t="inlineStr">
+      <c r="AA13" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2111,7 +2127,7 @@
         <f>IFERROR(P14/P11-1,"")</f>
         <v/>
       </c>
-      <c r="AA14" t="inlineStr">
+      <c r="AA14" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2190,7 +2206,7 @@
         <f>IFERROR(P15/P12-1,"")</f>
         <v/>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="AA15" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2269,7 +2285,7 @@
         <f>IFERROR(P16/P13-1,"")</f>
         <v/>
       </c>
-      <c r="AA16" t="inlineStr">
+      <c r="AA16" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2348,7 +2364,7 @@
         <f>IFERROR(P17/P14-1,"")</f>
         <v/>
       </c>
-      <c r="AA17" t="inlineStr">
+      <c r="AA17" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2427,7 +2443,7 @@
         <f>IFERROR(P18/P15-1,"")</f>
         <v/>
       </c>
-      <c r="AA18" t="inlineStr">
+      <c r="AA18" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2506,7 +2522,7 @@
         <f>IFERROR(P19/P16-1,"")</f>
         <v/>
       </c>
-      <c r="AA19" t="inlineStr">
+      <c r="AA19" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2585,7 +2601,7 @@
         <f>IFERROR(P20/P17-1,"")</f>
         <v/>
       </c>
-      <c r="AA20" t="inlineStr">
+      <c r="AA20" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2664,7 +2680,7 @@
         <f>IFERROR(P21/P18-1,"")</f>
         <v/>
       </c>
-      <c r="AA21" t="inlineStr">
+      <c r="AA21" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2743,7 +2759,7 @@
         <f>IFERROR(P22/P19-1,"")</f>
         <v/>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="AA22" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2822,7 +2838,7 @@
         <f>IFERROR(P23/P20-1,"")</f>
         <v/>
       </c>
-      <c r="AA23" t="inlineStr">
+      <c r="AA23" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2901,7 +2917,7 @@
         <f>IFERROR(P24/P21-1,"")</f>
         <v/>
       </c>
-      <c r="AA24" t="inlineStr">
+      <c r="AA24" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -2980,7 +2996,7 @@
         <f>IFERROR(P25/P22-1,"")</f>
         <v/>
       </c>
-      <c r="AA25" t="inlineStr">
+      <c r="AA25" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3059,7 +3075,7 @@
         <f>IFERROR(P26/P23-1,"")</f>
         <v/>
       </c>
-      <c r="AA26" t="inlineStr">
+      <c r="AA26" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3138,7 +3154,7 @@
         <f>IFERROR(P27/P24-1,"")</f>
         <v/>
       </c>
-      <c r="AA27" t="inlineStr">
+      <c r="AA27" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3217,7 +3233,7 @@
         <f>IFERROR(P28/P25-1,"")</f>
         <v/>
       </c>
-      <c r="AA28" t="inlineStr">
+      <c r="AA28" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3296,7 +3312,7 @@
         <f>IFERROR(P29/P26-1,"")</f>
         <v/>
       </c>
-      <c r="AA29" t="inlineStr">
+      <c r="AA29" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3375,7 +3391,7 @@
         <f>IFERROR(P30/P27-1,"")</f>
         <v/>
       </c>
-      <c r="AA30" t="inlineStr">
+      <c r="AA30" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3454,7 +3470,7 @@
         <f>IFERROR(P31/P28-1,"")</f>
         <v/>
       </c>
-      <c r="AA31" t="inlineStr">
+      <c r="AA31" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3533,7 +3549,7 @@
         <f>IFERROR(P32/P29-1,"")</f>
         <v/>
       </c>
-      <c r="AA32" t="inlineStr">
+      <c r="AA32" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3612,7 +3628,7 @@
         <f>IFERROR(P33/P30-1,"")</f>
         <v/>
       </c>
-      <c r="AA33" t="inlineStr">
+      <c r="AA33" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3696,7 +3712,7 @@
           <t>lsr_accum|stealth_grind|oi_ignition</t>
         </is>
       </c>
-      <c r="AA34" t="inlineStr">
+      <c r="AA34" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3785,7 +3801,7 @@
           <t>lsr_accum|stealth_grind|oi_ignition</t>
         </is>
       </c>
-      <c r="AA35" t="inlineStr">
+      <c r="AA35" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3850,7 +3866,7 @@
           <t>dist_wall|post_climax</t>
         </is>
       </c>
-      <c r="AA36" t="inlineStr">
+      <c r="AA36" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -3934,7 +3950,7 @@
         <f>IFERROR(P37/P34-1,"")</f>
         <v/>
       </c>
-      <c r="AA37" t="inlineStr">
+      <c r="AA37" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -4013,7 +4029,7 @@
         <f>IFERROR(P38/P35-1,"")</f>
         <v/>
       </c>
-      <c r="AA38" t="inlineStr">
+      <c r="AA38" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -4092,7 +4108,7 @@
         <f>IFERROR(P39/P36-1,"")</f>
         <v/>
       </c>
-      <c r="AA39" t="inlineStr">
+      <c r="AA39" s="27" t="inlineStr">
         <is>
           <t>Binance_spot</t>
         </is>
@@ -4107,6 +4123,345 @@
         <f>IF(OR(AB39="",D39="",D39=0),"",AB39/D39)</f>
         <v/>
       </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="58" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B40" s="59" t="n">
+        <v>0.056915</v>
+      </c>
+      <c r="C40" s="57" t="n">
+        <v>-0.09745231715678249</v>
+      </c>
+      <c r="D40" s="57" t="n">
+        <v>253304478</v>
+      </c>
+      <c r="E40" s="57" t="n">
+        <v>0.4804</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-0.000806</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-0.002363</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-0.000139</v>
+      </c>
+      <c r="I40" t="n">
+        <v>24</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>neg_batch</t>
+        </is>
+      </c>
+      <c r="K40" s="56" t="n"/>
+      <c r="L40" t="n">
+        <v>18027284</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.1805</v>
+      </c>
+      <c r="P40" t="n">
+        <v>2.0276</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.7996</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0.5822154271059381</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="56" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB40" s="57" t="n">
+        <v>19910000</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>0.462</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="58" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B41" s="59" t="n">
+        <v>0.047883</v>
+      </c>
+      <c r="C41" s="57" t="n">
+        <v>-0.1586927874901168</v>
+      </c>
+      <c r="D41" s="57" t="n">
+        <v>172554826</v>
+      </c>
+      <c r="E41" s="57" t="n">
+        <v>0.4791</v>
+      </c>
+      <c r="F41" t="n">
+        <v>-0.000349</v>
+      </c>
+      <c r="G41" t="n">
+        <v>-0.000722</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-9.66e-05</v>
+      </c>
+      <c r="I41" t="n">
+        <v>24</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>neg_light</t>
+        </is>
+      </c>
+      <c r="K41" s="56" t="n"/>
+      <c r="L41" t="n">
+        <v>17469390</v>
+      </c>
+      <c r="O41" t="n">
+        <v>1.3197</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2.2658</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>1.8843</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0.5824432871392003</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA41" s="56" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB41" s="57" t="n">
+        <v>12180000</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>0.493</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="58" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B42" s="59" t="n">
+        <v>0.043163</v>
+      </c>
+      <c r="C42" s="57" t="n">
+        <v>-0.09857360649917513</v>
+      </c>
+      <c r="D42" s="57" t="n">
+        <v>143022585</v>
+      </c>
+      <c r="E42" s="57" t="n">
+        <v>0.4883</v>
+      </c>
+      <c r="F42" t="n">
+        <v>-0.000186</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-0.000821</v>
+      </c>
+      <c r="H42" t="n">
+        <v>3.5e-06</v>
+      </c>
+      <c r="I42" t="n">
+        <v>24</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>neg_light</t>
+        </is>
+      </c>
+      <c r="K42" s="56" t="n"/>
+      <c r="L42" t="n">
+        <v>17252550</v>
+      </c>
+      <c r="O42" t="n">
+        <v>1.3123</v>
+      </c>
+      <c r="P42" t="n">
+        <v>2.1466</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1.7263</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0.6113388614553248</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="56" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB42" s="57" t="n">
+        <v>12350000</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>0.481</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="58" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B43" s="59" t="n">
+        <v>0.051353</v>
+      </c>
+      <c r="C43" s="57" t="n">
+        <v>0.1897458471375948</v>
+      </c>
+      <c r="D43" s="57" t="n">
+        <v>471564742</v>
+      </c>
+      <c r="E43" s="57" t="n">
+        <v>0.4906</v>
+      </c>
+      <c r="F43" t="n">
+        <v>-0.000548</v>
+      </c>
+      <c r="G43" t="n">
+        <v>-0.002347</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.25e-05</v>
+      </c>
+      <c r="I43" t="n">
+        <v>24</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>neg_batch</t>
+        </is>
+      </c>
+      <c r="K43" s="56" t="n"/>
+      <c r="L43" t="n">
+        <v>17356910</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1.3135</v>
+      </c>
+      <c r="P43" t="n">
+        <v>2.046</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1.649</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0.6419843597262952</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA43" s="56" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB43" s="57" t="n">
+        <v>46830000</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>0.483</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="60" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B44" s="61" t="n">
+        <v>0.0519</v>
+      </c>
+      <c r="C44" s="62" t="n">
+        <v>0.01065176328549455</v>
+      </c>
+      <c r="D44" s="62" t="n">
+        <v>102200000</v>
+      </c>
+      <c r="E44" s="62" t="n">
+        <v>0.486</v>
+      </c>
+      <c r="F44" s="63" t="n"/>
+      <c r="G44" s="63" t="n"/>
+      <c r="H44" s="63" t="n"/>
+      <c r="I44" s="63" t="n"/>
+      <c r="J44" s="63" t="inlineStr">
+        <is>
+          <t>near_zero</t>
+        </is>
+      </c>
+      <c r="K44" s="64" t="n"/>
+      <c r="L44" s="63" t="n">
+        <v>18070000</v>
+      </c>
+      <c r="M44" s="63" t="n"/>
+      <c r="N44" s="63" t="n"/>
+      <c r="O44" s="63" t="n">
+        <v>1.199</v>
+      </c>
+      <c r="P44" s="63" t="n"/>
+      <c r="Q44" s="63" t="n">
+        <v>1.396</v>
+      </c>
+      <c r="R44" s="63" t="n"/>
+      <c r="S44" s="63" t="n"/>
+      <c r="T44" s="63" t="n"/>
+      <c r="U44" s="63" t="n"/>
+      <c r="V44" s="63" t="n"/>
+      <c r="W44" s="63" t="n"/>
+      <c r="X44" s="63" t="n"/>
+      <c r="Y44" s="63" t="n"/>
+      <c r="Z44" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA44" s="64" t="inlineStr">
+        <is>
+          <t>Binance_spot</t>
+        </is>
+      </c>
+      <c r="AB44" s="62" t="n">
+        <v>6860000</v>
+      </c>
+      <c r="AC44" s="63" t="n">
+        <v>0.473</v>
+      </c>
+      <c r="AD44" s="63" t="n"/>
+      <c r="AE44" s="63" t="n"/>
+      <c r="AF44" s="63" t="n"/>
+      <c r="AG44" s="63" t="n"/>
+      <c r="AH44" s="63" t="n"/>
+      <c r="AI44" s="63" t="n"/>
+      <c r="AJ44" s="63" t="n"/>
+      <c r="AK44" s="63" t="n"/>
+      <c r="AL44" s="63" t="n"/>
+      <c r="AM44" s="63" t="n"/>
+      <c r="AN44" s="63" t="n"/>
+      <c r="AO44" s="63" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4551,6 +4906,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="53" t="inlineStr">
         <is>
@@ -4646,13 +5002,27 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="C5" s="33" t="n"/>
-      <c r="D5" s="33" t="n"/>
-      <c r="E5" s="33" t="n"/>
+      <c r="C5" s="65" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
+        <is>
+          <t>+31.3% vs T0=0.0377</t>
+        </is>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>Tu +897% dinh (0.672, 27/07 wick) ve +31.3%. advisor exit VWAP 0.1971 -&gt; px_now/exit = -74.9%. Crowd giu tui -73.4% tu exit.</t>
+        </is>
+      </c>
       <c r="F5" s="33" t="n"/>
       <c r="G5" s="33" t="n"/>
       <c r="H5" s="33" t="n"/>
-      <c r="I5" s="33" t="n"/>
+      <c r="I5" s="33" t="inlineStr">
+        <is>
+          <t>MUA_T0_DUNG — exit advisor 19-21/07 chuan xac</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="28">
       <c r="A6" s="32" t="inlineStr">

</xml_diff>

<commit_message>
backfill BANK/TAG/BR/IDOL tới 16/08; COOKIE/BROCCOLIF3B/KOMA ghi row nhưng VALIDATE_FAIL schema
BANK/TAG/BR/IDOL: lấp gap 14-16/08 (10-16/08 cho IDOL/BR) thành công, last=2026-08-16.
COOKIE/BROCCOLIF3B/KOMA: taker col mismatch (col8 header vs col5 EXPORT_COL_MAP) →
  validate_written_pack FAIL mỗi ngày. Data row được ghi nhưng schema sai. Nợ rebuild.
Guard dry-run 16/08: 0 STALE_GAP, 8 SKIP_EXISTS — đúng.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/case_files/CASE_BANK.xlsx
+++ b/docs/case_files/CASE_BANK.xlsx
@@ -993,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AO44"/>
+  <dimension ref="A1:AO51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="27" min="1" max="1"/>
@@ -4142,40 +4142,40 @@
       <c r="E40" s="57" t="n">
         <v>0.4804</v>
       </c>
-      <c r="F40" t="n">
+      <c r="F40" s="27" t="n">
         <v>-0.000806</v>
       </c>
-      <c r="G40" t="n">
+      <c r="G40" s="27" t="n">
         <v>-0.002363</v>
       </c>
-      <c r="H40" t="n">
+      <c r="H40" s="27" t="n">
         <v>-0.000139</v>
       </c>
-      <c r="I40" t="n">
+      <c r="I40" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40" s="27" t="inlineStr">
         <is>
           <t>neg_batch</t>
         </is>
       </c>
       <c r="K40" s="56" t="n"/>
-      <c r="L40" t="n">
+      <c r="L40" s="27" t="n">
         <v>18027284</v>
       </c>
-      <c r="O40" t="n">
+      <c r="O40" s="27" t="n">
         <v>1.1805</v>
       </c>
-      <c r="P40" t="n">
+      <c r="P40" s="27" t="n">
         <v>2.0276</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="Q40" s="27" t="n">
         <v>1.7996</v>
       </c>
-      <c r="R40" t="n">
+      <c r="R40" s="27" t="n">
         <v>0.5822154271059381</v>
       </c>
-      <c r="Z40" t="n">
+      <c r="Z40" s="27" t="n">
         <v>0</v>
       </c>
       <c r="AA40" s="56" t="inlineStr">
@@ -4186,7 +4186,7 @@
       <c r="AB40" s="57" t="n">
         <v>19910000</v>
       </c>
-      <c r="AC40" t="n">
+      <c r="AC40" s="27" t="n">
         <v>0.462</v>
       </c>
     </row>
@@ -4208,40 +4208,40 @@
       <c r="E41" s="57" t="n">
         <v>0.4791</v>
       </c>
-      <c r="F41" t="n">
+      <c r="F41" s="27" t="n">
         <v>-0.000349</v>
       </c>
-      <c r="G41" t="n">
+      <c r="G41" s="27" t="n">
         <v>-0.000722</v>
       </c>
-      <c r="H41" t="n">
+      <c r="H41" s="27" t="n">
         <v>-9.66e-05</v>
       </c>
-      <c r="I41" t="n">
+      <c r="I41" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" s="27" t="inlineStr">
         <is>
           <t>neg_light</t>
         </is>
       </c>
       <c r="K41" s="56" t="n"/>
-      <c r="L41" t="n">
+      <c r="L41" s="27" t="n">
         <v>17469390</v>
       </c>
-      <c r="O41" t="n">
+      <c r="O41" s="27" t="n">
         <v>1.3197</v>
       </c>
-      <c r="P41" t="n">
+      <c r="P41" s="27" t="n">
         <v>2.2658</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="Q41" s="27" t="n">
         <v>1.8843</v>
       </c>
-      <c r="R41" t="n">
+      <c r="R41" s="27" t="n">
         <v>0.5824432871392003</v>
       </c>
-      <c r="Z41" t="n">
+      <c r="Z41" s="27" t="n">
         <v>0</v>
       </c>
       <c r="AA41" s="56" t="inlineStr">
@@ -4252,7 +4252,7 @@
       <c r="AB41" s="57" t="n">
         <v>12180000</v>
       </c>
-      <c r="AC41" t="n">
+      <c r="AC41" s="27" t="n">
         <v>0.493</v>
       </c>
     </row>
@@ -4274,40 +4274,40 @@
       <c r="E42" s="57" t="n">
         <v>0.4883</v>
       </c>
-      <c r="F42" t="n">
+      <c r="F42" s="27" t="n">
         <v>-0.000186</v>
       </c>
-      <c r="G42" t="n">
+      <c r="G42" s="27" t="n">
         <v>-0.000821</v>
       </c>
-      <c r="H42" t="n">
+      <c r="H42" s="27" t="n">
         <v>3.5e-06</v>
       </c>
-      <c r="I42" t="n">
+      <c r="I42" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="27" t="inlineStr">
         <is>
           <t>neg_light</t>
         </is>
       </c>
       <c r="K42" s="56" t="n"/>
-      <c r="L42" t="n">
+      <c r="L42" s="27" t="n">
         <v>17252550</v>
       </c>
-      <c r="O42" t="n">
+      <c r="O42" s="27" t="n">
         <v>1.3123</v>
       </c>
-      <c r="P42" t="n">
+      <c r="P42" s="27" t="n">
         <v>2.1466</v>
       </c>
-      <c r="Q42" t="n">
+      <c r="Q42" s="27" t="n">
         <v>1.7263</v>
       </c>
-      <c r="R42" t="n">
+      <c r="R42" s="27" t="n">
         <v>0.6113388614553248</v>
       </c>
-      <c r="Z42" t="n">
+      <c r="Z42" s="27" t="n">
         <v>0</v>
       </c>
       <c r="AA42" s="56" t="inlineStr">
@@ -4318,7 +4318,7 @@
       <c r="AB42" s="57" t="n">
         <v>12350000</v>
       </c>
-      <c r="AC42" t="n">
+      <c r="AC42" s="27" t="n">
         <v>0.481</v>
       </c>
     </row>
@@ -4340,40 +4340,40 @@
       <c r="E43" s="57" t="n">
         <v>0.4906</v>
       </c>
-      <c r="F43" t="n">
+      <c r="F43" s="27" t="n">
         <v>-0.000548</v>
       </c>
-      <c r="G43" t="n">
+      <c r="G43" s="27" t="n">
         <v>-0.002347</v>
       </c>
-      <c r="H43" t="n">
+      <c r="H43" s="27" t="n">
         <v>1.25e-05</v>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="27" t="inlineStr">
         <is>
           <t>neg_batch</t>
         </is>
       </c>
       <c r="K43" s="56" t="n"/>
-      <c r="L43" t="n">
+      <c r="L43" s="27" t="n">
         <v>17356910</v>
       </c>
-      <c r="O43" t="n">
+      <c r="O43" s="27" t="n">
         <v>1.3135</v>
       </c>
-      <c r="P43" t="n">
+      <c r="P43" s="27" t="n">
         <v>2.046</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="Q43" s="27" t="n">
         <v>1.649</v>
       </c>
-      <c r="R43" t="n">
+      <c r="R43" s="27" t="n">
         <v>0.6419843597262952</v>
       </c>
-      <c r="Z43" t="n">
+      <c r="Z43" s="27" t="n">
         <v>0</v>
       </c>
       <c r="AA43" s="56" t="inlineStr">
@@ -4384,7 +4384,7 @@
       <c r="AB43" s="57" t="n">
         <v>46830000</v>
       </c>
-      <c r="AC43" t="n">
+      <c r="AC43" s="27" t="n">
         <v>0.483</v>
       </c>
     </row>
@@ -4462,6 +4462,482 @@
       <c r="AM44" s="63" t="n"/>
       <c r="AN44" s="63" t="n"/>
       <c r="AO44" s="63" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B45" s="27" t="n">
+        <v>0.0404143452896341</v>
+      </c>
+      <c r="C45" s="27">
+        <f>IFERROR(B45/B44-1,"")</f>
+        <v/>
+      </c>
+      <c r="D45" s="27" t="n">
+        <v>140686649.01256</v>
+      </c>
+      <c r="E45" s="27" t="n">
+        <v>47.657681</v>
+      </c>
+      <c r="F45" s="27" t="n">
+        <v>4.8475e-05</v>
+      </c>
+      <c r="G45" s="27" t="n">
+        <v>4.416e-05</v>
+      </c>
+      <c r="H45" s="27" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I45" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L45" s="27" t="n">
+        <v>12984678.97891008</v>
+      </c>
+      <c r="O45" s="27" t="n">
+        <v>1.5928</v>
+      </c>
+      <c r="P45" s="27" t="n">
+        <v>1.8433</v>
+      </c>
+      <c r="Q45" s="27" t="n">
+        <v>1.4295</v>
+      </c>
+      <c r="R45" s="27">
+        <f>IFERROR(O45/P45,"")</f>
+        <v/>
+      </c>
+      <c r="S45" s="27">
+        <f>IFERROR(AVERAGE(R43:R45),"")</f>
+        <v/>
+      </c>
+      <c r="T45" s="27">
+        <f>IFERROR(Q45/Q40,"")</f>
+        <v/>
+      </c>
+      <c r="U45" s="27">
+        <f>IFERROR(O45/O42-1,"")</f>
+        <v/>
+      </c>
+      <c r="V45" s="27">
+        <f>IFERROR(P45/P42-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ45" s="27">
+        <f>IF(OR(AB45="",D45="",D45=0),"",AB45/D45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B46" s="27" t="n">
+        <v>0.0389331582839826</v>
+      </c>
+      <c r="C46" s="27">
+        <f>IFERROR(B46/B45-1,"")</f>
+        <v/>
+      </c>
+      <c r="D46" s="27" t="n">
+        <v>42263053.84667</v>
+      </c>
+      <c r="E46" s="27" t="n">
+        <v>49.246308</v>
+      </c>
+      <c r="F46" s="27" t="n">
+        <v>-9.721166666666668e-05</v>
+      </c>
+      <c r="G46" s="27" t="n">
+        <v>-0.00029585</v>
+      </c>
+      <c r="H46" s="27" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I46" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L46" s="27" t="n">
+        <v>13196123.73636998</v>
+      </c>
+      <c r="O46" s="27" t="n">
+        <v>1.4526</v>
+      </c>
+      <c r="P46" s="27" t="n">
+        <v>1.9412</v>
+      </c>
+      <c r="Q46" s="27" t="n">
+        <v>1.4498</v>
+      </c>
+      <c r="R46" s="27">
+        <f>IFERROR(O46/P46,"")</f>
+        <v/>
+      </c>
+      <c r="S46" s="27">
+        <f>IFERROR(AVERAGE(R44:R46),"")</f>
+        <v/>
+      </c>
+      <c r="T46" s="27">
+        <f>IFERROR(Q46/Q41,"")</f>
+        <v/>
+      </c>
+      <c r="U46" s="27">
+        <f>IFERROR(O46/O43-1,"")</f>
+        <v/>
+      </c>
+      <c r="V46" s="27">
+        <f>IFERROR(P46/P43-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ46" s="27">
+        <f>IF(OR(AB46="",D46="",D46=0),"",AB46/D46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B47" s="27" t="n">
+        <v>0.0373057526039732</v>
+      </c>
+      <c r="C47" s="27">
+        <f>IFERROR(B47/B46-1,"")</f>
+        <v/>
+      </c>
+      <c r="D47" s="27" t="n">
+        <v>45394765.99188</v>
+      </c>
+      <c r="E47" s="27" t="n">
+        <v>46.007235</v>
+      </c>
+      <c r="F47" s="27" t="n">
+        <v>-8.702333333333332e-05</v>
+      </c>
+      <c r="G47" s="27" t="n">
+        <v>-0.00030814</v>
+      </c>
+      <c r="H47" s="27" t="n">
+        <v>3.123e-05</v>
+      </c>
+      <c r="I47" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L47" s="27" t="n">
+        <v>13337814.73104</v>
+      </c>
+      <c r="O47" s="27" t="n">
+        <v>1.5683</v>
+      </c>
+      <c r="P47" s="27" t="n">
+        <v>2.0469</v>
+      </c>
+      <c r="Q47" s="27" t="n">
+        <v>1.5813</v>
+      </c>
+      <c r="R47" s="27">
+        <f>IFERROR(O47/P47,"")</f>
+        <v/>
+      </c>
+      <c r="S47" s="27">
+        <f>IFERROR(AVERAGE(R45:R47),"")</f>
+        <v/>
+      </c>
+      <c r="T47" s="27">
+        <f>IFERROR(Q47/Q42,"")</f>
+        <v/>
+      </c>
+      <c r="U47" s="27">
+        <f>IFERROR(O47/O44-1,"")</f>
+        <v/>
+      </c>
+      <c r="V47" s="27">
+        <f>IFERROR(P47/P44-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ47" s="27">
+        <f>IF(OR(AB47="",D47="",D47=0),"",AB47/D47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B48" s="27" t="n">
+        <v>0.0363926583940916</v>
+      </c>
+      <c r="C48" s="27">
+        <f>IFERROR(B48/B47-1,"")</f>
+        <v/>
+      </c>
+      <c r="D48" s="27" t="n">
+        <v>54495385.01868</v>
+      </c>
+      <c r="E48" s="27" t="n">
+        <v>48.408399</v>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>-0.000389125</v>
+      </c>
+      <c r="G48" s="27" t="n">
+        <v>-0.00084272</v>
+      </c>
+      <c r="H48" s="27" t="n">
+        <v>6.02e-06</v>
+      </c>
+      <c r="I48" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L48" s="27" t="n">
+        <v>11832075.85119</v>
+      </c>
+      <c r="O48" s="27" t="n">
+        <v>1.5795</v>
+      </c>
+      <c r="P48" s="27" t="n">
+        <v>1.907</v>
+      </c>
+      <c r="Q48" s="27" t="n">
+        <v>1.3883</v>
+      </c>
+      <c r="R48" s="27">
+        <f>IFERROR(O48/P48,"")</f>
+        <v/>
+      </c>
+      <c r="S48" s="27">
+        <f>IFERROR(AVERAGE(R46:R48),"")</f>
+        <v/>
+      </c>
+      <c r="T48" s="27">
+        <f>IFERROR(Q48/Q43,"")</f>
+        <v/>
+      </c>
+      <c r="U48" s="27">
+        <f>IFERROR(O48/O45-1,"")</f>
+        <v/>
+      </c>
+      <c r="V48" s="27">
+        <f>IFERROR(P48/P45-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ48" s="27">
+        <f>IF(OR(AB48="",D48="",D48=0),"",AB48/D48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="n">
+        <v>0.0373570870676163</v>
+      </c>
+      <c r="C49" s="27">
+        <f>IFERROR(B49/B48-1,"")</f>
+        <v/>
+      </c>
+      <c r="D49" s="27" t="n">
+        <v>43707076.14468</v>
+      </c>
+      <c r="E49" s="27" t="n">
+        <v>48.253558</v>
+      </c>
+      <c r="F49" s="27" t="n">
+        <v>1.937e-05</v>
+      </c>
+      <c r="G49" s="27" t="n">
+        <v>-7.900000000000001e-06</v>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I49" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L49" s="27" t="n">
+        <v>11813030.8373</v>
+      </c>
+      <c r="O49" s="27" t="n">
+        <v>1.559</v>
+      </c>
+      <c r="P49" s="27" t="n">
+        <v>1.8662</v>
+      </c>
+      <c r="Q49" s="27" t="n">
+        <v>1.4462</v>
+      </c>
+      <c r="R49" s="27">
+        <f>IFERROR(O49/P49,"")</f>
+        <v/>
+      </c>
+      <c r="S49" s="27">
+        <f>IFERROR(AVERAGE(R47:R49),"")</f>
+        <v/>
+      </c>
+      <c r="T49" s="27">
+        <f>IFERROR(Q49/Q44,"")</f>
+        <v/>
+      </c>
+      <c r="U49" s="27">
+        <f>IFERROR(O49/O46-1,"")</f>
+        <v/>
+      </c>
+      <c r="V49" s="27">
+        <f>IFERROR(P49/P46-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ49" s="27">
+        <f>IF(OR(AB49="",D49="",D49=0),"",AB49/D49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B50" s="27" t="n">
+        <v>0.0375901118292134</v>
+      </c>
+      <c r="C50" s="27">
+        <f>IFERROR(B50/B49-1,"")</f>
+        <v/>
+      </c>
+      <c r="D50" s="27" t="n">
+        <v>28138687.39511</v>
+      </c>
+      <c r="E50" s="27" t="n">
+        <v>47.210051</v>
+      </c>
+      <c r="F50" s="27" t="n">
+        <v>4.253166666666667e-05</v>
+      </c>
+      <c r="G50" s="27" t="n">
+        <v>5.19e-06</v>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I50" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="L50" s="27" t="n">
+        <v>11699705.86807</v>
+      </c>
+      <c r="O50" s="27" t="n">
+        <v>1.593</v>
+      </c>
+      <c r="P50" s="27" t="n">
+        <v>1.7824</v>
+      </c>
+      <c r="Q50" s="27" t="n">
+        <v>1.3838</v>
+      </c>
+      <c r="R50" s="27">
+        <f>IFERROR(O50/P50,"")</f>
+        <v/>
+      </c>
+      <c r="S50" s="27">
+        <f>IFERROR(AVERAGE(R48:R50),"")</f>
+        <v/>
+      </c>
+      <c r="T50" s="27">
+        <f>IFERROR(Q50/Q45,"")</f>
+        <v/>
+      </c>
+      <c r="U50" s="27">
+        <f>IFERROR(O50/O47-1,"")</f>
+        <v/>
+      </c>
+      <c r="V50" s="27">
+        <f>IFERROR(P50/P47-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ50" s="27">
+        <f>IF(OR(AB50="",D50="",D50=0),"",AB50/D50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.03635792928012117</v>
+      </c>
+      <c r="C51">
+        <f>IFERROR(B51/B50-1,"")</f>
+        <v/>
+      </c>
+      <c r="D51" t="n">
+        <v>19287848.72461</v>
+      </c>
+      <c r="E51" t="n">
+        <v>46.141003</v>
+      </c>
+      <c r="F51" t="n">
+        <v>2.4445e-05</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-4.002e-05</v>
+      </c>
+      <c r="H51" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="I51" t="n">
+        <v>6</v>
+      </c>
+      <c r="L51" t="n">
+        <v>11251300.09384519</v>
+      </c>
+      <c r="O51" t="n">
+        <v>1.6943</v>
+      </c>
+      <c r="P51" t="n">
+        <v>1.8466</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>1.4015</v>
+      </c>
+      <c r="R51">
+        <f>IFERROR(O51/P51,"")</f>
+        <v/>
+      </c>
+      <c r="S51">
+        <f>IFERROR(AVERAGE(R49:R51),"")</f>
+        <v/>
+      </c>
+      <c r="T51">
+        <f>IFERROR(Q51/Q46,"")</f>
+        <v/>
+      </c>
+      <c r="U51">
+        <f>IFERROR(O51/O48-1,"")</f>
+        <v/>
+      </c>
+      <c r="V51">
+        <f>IFERROR(P51/P48-1,"")</f>
+        <v/>
+      </c>
+      <c r="AJ51">
+        <f>IF(OR(AB51="",D51="",D51=0),"",AB51/D51)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4906,7 +5382,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="28">
       <c r="A3" s="53" t="inlineStr">
         <is>

</xml_diff>